<commit_message>
Enrichissements : PPR + noms arabes + téléphone (enseignants & élèves, appel parent au dépassement du seuil), rapport enseignant A4 police arabique 10pt avec 6 modèles prêts bilingues, grille horaire export Excel/CSV compatible import + synchro tables de service, fix jours arabes à hamza
</commit_message>
<xml_diff>
--- a/public/templates/ListEleve_20260905.xlsx
+++ b/public/templates/ListEleve_20260905.xlsx
@@ -397,13 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:H13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,9 +420,18 @@
         <v>Prénom</v>
       </c>
       <c r="D1" t="str">
+        <v>Nom (arabe)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Prénom (arabe)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Téléphone parent</v>
+      </c>
+      <c r="G1" t="str">
         <v>Classe</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>Niveau</v>
       </c>
     </row>
@@ -434,9 +446,18 @@
         <v>Youssef</v>
       </c>
       <c r="D2" t="str">
+        <v>العلوي</v>
+      </c>
+      <c r="E2" t="str">
+        <v>يوسف</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0661234501</v>
+      </c>
+      <c r="G2" t="str">
         <v>TCSF-1</v>
       </c>
-      <c r="E2" t="str">
+      <c r="H2" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -451,9 +472,18 @@
         <v>Aya</v>
       </c>
       <c r="D3" t="str">
+        <v>بنجلون</v>
+      </c>
+      <c r="E3" t="str">
+        <v>آية</v>
+      </c>
+      <c r="F3" t="str">
+        <v>0661234502</v>
+      </c>
+      <c r="G3" t="str">
         <v>TCSF-1</v>
       </c>
-      <c r="E3" t="str">
+      <c r="H3" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -468,9 +498,18 @@
         <v>Omar</v>
       </c>
       <c r="D4" t="str">
+        <v>الشكيري</v>
+      </c>
+      <c r="E4" t="str">
+        <v>عمر</v>
+      </c>
+      <c r="F4" t="str">
+        <v>0661234503</v>
+      </c>
+      <c r="G4" t="str">
         <v>TCSF-1</v>
       </c>
-      <c r="E4" t="str">
+      <c r="H4" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -485,9 +524,18 @@
         <v>Salma</v>
       </c>
       <c r="D5" t="str">
+        <v>الدويري</v>
+      </c>
+      <c r="E5" t="str">
+        <v>سلمى</v>
+      </c>
+      <c r="F5" t="str">
+        <v>0661234504</v>
+      </c>
+      <c r="G5" t="str">
         <v>TCSF-1</v>
       </c>
-      <c r="E5" t="str">
+      <c r="H5" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -502,9 +550,18 @@
         <v>Mehdi</v>
       </c>
       <c r="D6" t="str">
+        <v>العمراني</v>
+      </c>
+      <c r="E6" t="str">
+        <v>مهدي</v>
+      </c>
+      <c r="F6" t="str">
+        <v>0661234505</v>
+      </c>
+      <c r="G6" t="str">
         <v>TCSF-2</v>
       </c>
-      <c r="E6" t="str">
+      <c r="H6" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -519,9 +576,18 @@
         <v>Nadia</v>
       </c>
       <c r="D7" t="str">
+        <v>الفاروقي</v>
+      </c>
+      <c r="E7" t="str">
+        <v>نادية</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0661234506</v>
+      </c>
+      <c r="G7" t="str">
         <v>TCSF-2</v>
       </c>
-      <c r="E7" t="str">
+      <c r="H7" t="str">
         <v>Tronc Commun</v>
       </c>
     </row>
@@ -536,9 +602,18 @@
         <v>Hamza</v>
       </c>
       <c r="D8" t="str">
+        <v>الغالي</v>
+      </c>
+      <c r="E8" t="str">
+        <v>حمزة</v>
+      </c>
+      <c r="F8" t="str">
+        <v>0661234507</v>
+      </c>
+      <c r="G8" t="str">
         <v>1BACSC-1</v>
       </c>
-      <c r="E8" t="str">
+      <c r="H8" t="str">
         <v>1ère Année Bac</v>
       </c>
     </row>
@@ -553,9 +628,18 @@
         <v>Imane</v>
       </c>
       <c r="D9" t="str">
+        <v>الحساني</v>
+      </c>
+      <c r="E9" t="str">
+        <v>إيمان</v>
+      </c>
+      <c r="F9" t="str">
+        <v>0661234508</v>
+      </c>
+      <c r="G9" t="str">
         <v>1BACSC-1</v>
       </c>
-      <c r="E9" t="str">
+      <c r="H9" t="str">
         <v>1ère Année Bac</v>
       </c>
     </row>
@@ -570,9 +654,18 @@
         <v>Karim</v>
       </c>
       <c r="D10" t="str">
+        <v>الإدريسي</v>
+      </c>
+      <c r="E10" t="str">
+        <v>كريم</v>
+      </c>
+      <c r="F10" t="str">
+        <v>0661234509</v>
+      </c>
+      <c r="G10" t="str">
         <v>2BACPC-1</v>
       </c>
-      <c r="E10" t="str">
+      <c r="H10" t="str">
         <v>2ème Année Bac</v>
       </c>
     </row>
@@ -587,9 +680,18 @@
         <v>Laila</v>
       </c>
       <c r="D11" t="str">
+        <v>الجاعيدي</v>
+      </c>
+      <c r="E11" t="str">
+        <v>ليلى</v>
+      </c>
+      <c r="F11" t="str">
+        <v>0661234510</v>
+      </c>
+      <c r="G11" t="str">
         <v>2BACPC-1</v>
       </c>
-      <c r="E11" t="str">
+      <c r="H11" t="str">
         <v>2ème Année Bac</v>
       </c>
     </row>
@@ -604,9 +706,18 @@
         <v>Adam</v>
       </c>
       <c r="D12" t="str">
+        <v>الكتاني</v>
+      </c>
+      <c r="E12" t="str">
+        <v>آدم</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0661234511</v>
+      </c>
+      <c r="G12" t="str">
         <v>2BACPC-2</v>
       </c>
-      <c r="E12" t="str">
+      <c r="H12" t="str">
         <v>2ème Année Bac</v>
       </c>
     </row>
@@ -621,15 +732,24 @@
         <v>Sofia</v>
       </c>
       <c r="D13" t="str">
+        <v>العمراني</v>
+      </c>
+      <c r="E13" t="str">
+        <v>صوفيا</v>
+      </c>
+      <c r="F13" t="str">
+        <v>0661234512</v>
+      </c>
+      <c r="G13" t="str">
         <v>2BACPC-2</v>
       </c>
-      <c r="E13" t="str">
+      <c r="H13" t="str">
         <v>2ème Année Bac</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>